<commit_message>
FY25 Review thermostat charts from Test.xlsx; playbook responsive fixes
- Parse FY23–FY25 thermostat grids from Test.xlsx; export JSON and wire Digital Platform charts via hook + dev middleware polling.
- Run fy25 thermostat export from export-roadmaps; add npm run export-fy25-review-charts.
- Allow main playbook column to shrink (min-width: 0); stack dual FY charts below 900px.

Made-with: Cursor
</commit_message>
<xml_diff>
--- a/Test.xlsx
+++ b/Test.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29912"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10817"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://goodmanglobal-my.sharepoint.com/personal/smithlx2_daikincomfort_com/Documents/Documents/LS-VP Strategic Marketing/Controls/DOCS Progress Reports/DOCS Financials/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/vishwas/Documents/DevelopmentProjects/Skyport-Web/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{EDAF8627-B7D0-4AFA-AF3E-4E5D1F0B8E68}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8B582EC6-B1DB-1649-9DDA-EA1C085766D4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-18780" yWindow="-20140" windowWidth="30240" windowHeight="17460" firstSheet="2" activeTab="5" xr2:uid="{564A4D30-3E13-E04F-96B0-B8BA94B7A041}"/>
+    <workbookView xWindow="23940" yWindow="1380" windowWidth="30240" windowHeight="18880" firstSheet="2" activeTab="3" xr2:uid="{564A4D30-3E13-E04F-96B0-B8BA94B7A041}"/>
   </bookViews>
   <sheets>
     <sheet name="OnBase Coding" sheetId="7" r:id="rId1"/>
@@ -448,12 +448,13 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="3">
+  <numFmts count="4">
+    <numFmt numFmtId="8" formatCode="&quot;$&quot;#,##0.00_);[Red]\(&quot;$&quot;#,##0.00\)"/>
     <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="164" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
   </numFmts>
-  <fonts count="13">
+  <fonts count="13" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -545,7 +546,7 @@
       <sz val="11"/>
       <color rgb="FF242424"/>
       <name val="Consolas"/>
-      <charset val="1"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="10">
@@ -1239,7 +1240,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="152">
+  <cellXfs count="153">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1454,6 +1455,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="8" fontId="0" fillId="2" borderId="7" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
@@ -5247,9 +5249,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -5287,7 +5289,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -5393,7 +5395,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -5535,7 +5537,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -5568,16 +5570,16 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4AC81046-4639-234D-87CF-6D2D04141E00}">
   <dimension ref="B1:J14"/>
-  <sheetFormatPr defaultColWidth="10.85546875" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="5.85546875" style="5" customWidth="1"/>
+    <col min="1" max="1" width="5.83203125" style="5" customWidth="1"/>
     <col min="2" max="2" width="12" style="5" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="49.28515625" style="5" bestFit="1" customWidth="1"/>
-    <col min="4" max="16384" width="10.85546875" style="5"/>
+    <col min="3" max="3" width="49.33203125" style="5" bestFit="1" customWidth="1"/>
+    <col min="4" max="16384" width="10.83203125" style="5"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:10" ht="15.95" thickBot="1"/>
-    <row r="2" spans="2:10" ht="15.95" thickBot="1">
+    <row r="1" spans="2:10" ht="16" thickBot="1" x14ac:dyDescent="0.25"/>
+    <row r="2" spans="2:10" ht="16" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B2" s="104" t="s">
         <v>0</v>
       </c>
@@ -5591,7 +5593,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="2:10">
+    <row r="3" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B3" s="107" t="s">
         <v>4</v>
       </c>
@@ -5605,7 +5607,7 @@
         <v>76410</v>
       </c>
     </row>
-    <row r="4" spans="2:10" ht="15.95" thickBot="1">
+    <row r="4" spans="2:10" ht="16" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B4" s="109" t="s">
         <v>6</v>
       </c>
@@ -5619,17 +5621,17 @@
         <v>50075</v>
       </c>
     </row>
-    <row r="12" spans="2:10">
+    <row r="12" spans="2:10" x14ac:dyDescent="0.2">
       <c r="D12" s="5">
         <v>220</v>
       </c>
     </row>
-    <row r="13" spans="2:10">
+    <row r="13" spans="2:10" x14ac:dyDescent="0.2">
       <c r="C13" s="5">
         <v>3</v>
       </c>
     </row>
-    <row r="14" spans="2:10">
+    <row r="14" spans="2:10" x14ac:dyDescent="0.2">
       <c r="J14" s="5">
         <v>7</v>
       </c>
@@ -5642,17 +5644,17 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{27AF65B5-FF90-5149-85EB-40A9651F80A1}">
   <dimension ref="B2:E11"/>
-  <sheetFormatPr defaultColWidth="10.85546875" defaultRowHeight="15.95"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="3.85546875" style="113" customWidth="1"/>
-    <col min="2" max="2" width="4.42578125" style="113" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="59.42578125" style="113" customWidth="1"/>
-    <col min="4" max="4" width="124.7109375" style="113" customWidth="1"/>
-    <col min="5" max="5" width="58.85546875" style="113" bestFit="1" customWidth="1"/>
-    <col min="6" max="16384" width="10.85546875" style="113"/>
+    <col min="1" max="1" width="3.83203125" style="113" customWidth="1"/>
+    <col min="2" max="2" width="4.5" style="113" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="59.5" style="113" customWidth="1"/>
+    <col min="4" max="4" width="124.6640625" style="113" customWidth="1"/>
+    <col min="5" max="5" width="58.83203125" style="113" bestFit="1" customWidth="1"/>
+    <col min="6" max="16384" width="10.83203125" style="113"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:5">
+    <row r="2" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B2" s="114" t="s">
         <v>88</v>
       </c>
@@ -5666,7 +5668,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="3" spans="2:5" ht="33.950000000000003">
+    <row r="3" spans="2:5" ht="34" x14ac:dyDescent="0.2">
       <c r="B3" s="120" t="s">
         <v>91</v>
       </c>
@@ -5680,7 +5682,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="4" spans="2:5" ht="33.950000000000003">
+    <row r="4" spans="2:5" ht="34" x14ac:dyDescent="0.2">
       <c r="B4" s="115" t="s">
         <v>94</v>
       </c>
@@ -5692,7 +5694,7 @@
       </c>
       <c r="E4" s="115"/>
     </row>
-    <row r="5" spans="2:5">
+    <row r="5" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B5" s="120" t="s">
         <v>96</v>
       </c>
@@ -5704,7 +5706,7 @@
       </c>
       <c r="E5" s="120"/>
     </row>
-    <row r="6" spans="2:5">
+    <row r="6" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B6" s="115" t="s">
         <v>98</v>
       </c>
@@ -5716,7 +5718,7 @@
       </c>
       <c r="E6" s="115"/>
     </row>
-    <row r="7" spans="2:5">
+    <row r="7" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B7" s="120" t="s">
         <v>100</v>
       </c>
@@ -5728,7 +5730,7 @@
       </c>
       <c r="E7" s="120"/>
     </row>
-    <row r="8" spans="2:5">
+    <row r="8" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B8" s="115" t="s">
         <v>102</v>
       </c>
@@ -5740,7 +5742,7 @@
       </c>
       <c r="E8" s="115"/>
     </row>
-    <row r="9" spans="2:5" ht="51">
+    <row r="9" spans="2:5" ht="51" x14ac:dyDescent="0.2">
       <c r="B9" s="120" t="s">
         <v>104</v>
       </c>
@@ -5754,7 +5756,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="10" spans="2:5" ht="76.5" customHeight="1">
+    <row r="10" spans="2:5" ht="76.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B10" s="115" t="s">
         <v>107</v>
       </c>
@@ -5768,7 +5770,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="11" spans="2:5" ht="135.94999999999999">
+    <row r="11" spans="2:5" ht="136" x14ac:dyDescent="0.2">
       <c r="B11" s="117" t="s">
         <v>110</v>
       </c>
@@ -5793,24 +5795,24 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{357ECBC5-E9B3-A941-BF6D-EA2F182E69DF}">
   <dimension ref="B1:O16"/>
-  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.5" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="2" max="2" width="17.85546875" customWidth="1"/>
-    <col min="3" max="9" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.7109375" customWidth="1"/>
-    <col min="11" max="11" width="13.140625" customWidth="1"/>
-    <col min="12" max="12" width="12.85546875" customWidth="1"/>
-    <col min="15" max="15" width="14.140625" customWidth="1"/>
+    <col min="2" max="2" width="17.83203125" customWidth="1"/>
+    <col min="3" max="9" width="12.1640625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.6640625" customWidth="1"/>
+    <col min="11" max="11" width="13.1640625" customWidth="1"/>
+    <col min="12" max="12" width="12.83203125" customWidth="1"/>
+    <col min="15" max="15" width="14.1640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:15">
+    <row r="1" spans="2:15" x14ac:dyDescent="0.2">
       <c r="C1" s="61">
         <f>'FY25'!B1</f>
         <v>447756</v>
       </c>
     </row>
-    <row r="2" spans="2:15" ht="15.95" thickBot="1"/>
-    <row r="3" spans="2:15" ht="15.95" thickBot="1">
+    <row r="2" spans="2:15" ht="16" thickBot="1" x14ac:dyDescent="0.25"/>
+    <row r="3" spans="2:15" ht="16" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B3" s="1"/>
       <c r="C3" s="74" t="s">
         <v>8</v>
@@ -5852,7 +5854,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="4" spans="2:15" hidden="1">
+    <row r="4" spans="2:15" hidden="1" x14ac:dyDescent="0.2">
       <c r="B4" s="127" t="s">
         <v>21</v>
       </c>
@@ -5889,7 +5891,7 @@
         <v>125529</v>
       </c>
     </row>
-    <row r="5" spans="2:15" hidden="1">
+    <row r="5" spans="2:15" hidden="1" x14ac:dyDescent="0.2">
       <c r="B5" s="129" t="s">
         <v>22</v>
       </c>
@@ -5943,7 +5945,7 @@
       </c>
       <c r="O5" s="128"/>
     </row>
-    <row r="6" spans="2:15" hidden="1">
+    <row r="6" spans="2:15" hidden="1" x14ac:dyDescent="0.2">
       <c r="B6" s="129" t="s">
         <v>23</v>
       </c>
@@ -5977,7 +5979,7 @@
       <c r="N6" s="134"/>
       <c r="O6" s="128"/>
     </row>
-    <row r="7" spans="2:15">
+    <row r="7" spans="2:15" x14ac:dyDescent="0.2">
       <c r="B7" s="129" t="s">
         <v>24</v>
       </c>
@@ -6022,7 +6024,7 @@
         <v>382021.14999999997</v>
       </c>
     </row>
-    <row r="8" spans="2:15">
+    <row r="8" spans="2:15" x14ac:dyDescent="0.2">
       <c r="B8" s="129" t="s">
         <v>25</v>
       </c>
@@ -6063,7 +6065,7 @@
         <v>1128965.6099999999</v>
       </c>
     </row>
-    <row r="9" spans="2:15">
+    <row r="9" spans="2:15" x14ac:dyDescent="0.2">
       <c r="B9" s="129" t="s">
         <v>26</v>
       </c>
@@ -6120,7 +6122,7 @@
         <v>1510986.7599999998</v>
       </c>
     </row>
-    <row r="10" spans="2:15" hidden="1">
+    <row r="10" spans="2:15" hidden="1" x14ac:dyDescent="0.2">
       <c r="B10" s="129" t="s">
         <v>27</v>
       </c>
@@ -6174,7 +6176,7 @@
       </c>
       <c r="O10" s="132"/>
     </row>
-    <row r="11" spans="2:15" hidden="1">
+    <row r="11" spans="2:15" hidden="1" x14ac:dyDescent="0.2">
       <c r="B11" s="129" t="s">
         <v>28</v>
       </c>
@@ -6228,7 +6230,7 @@
       </c>
       <c r="O11" s="131"/>
     </row>
-    <row r="12" spans="2:15" hidden="1">
+    <row r="12" spans="2:15" hidden="1" x14ac:dyDescent="0.2">
       <c r="B12" s="129" t="s">
         <v>29</v>
       </c>
@@ -6282,7 +6284,7 @@
       </c>
       <c r="O12" s="131"/>
     </row>
-    <row r="13" spans="2:15" hidden="1">
+    <row r="13" spans="2:15" hidden="1" x14ac:dyDescent="0.2">
       <c r="B13" s="129" t="s">
         <v>30</v>
       </c>
@@ -6336,7 +6338,7 @@
       </c>
       <c r="O13" s="132"/>
     </row>
-    <row r="15" spans="2:15">
+    <row r="15" spans="2:15" x14ac:dyDescent="0.2">
       <c r="B15" t="s">
         <v>31</v>
       </c>
@@ -6380,7 +6382,7 @@
         <v>1.3575569830240879</v>
       </c>
     </row>
-    <row r="16" spans="2:15">
+    <row r="16" spans="2:15" x14ac:dyDescent="0.2">
       <c r="B16" t="s">
         <v>32</v>
       </c>
@@ -6432,17 +6434,17 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AEEDF41F-1FC9-4176-ABE5-41DD99DA4F1F}">
   <dimension ref="A1:T27"/>
-  <sheetFormatPr defaultColWidth="10.85546875" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="43.42578125" style="5" bestFit="1" customWidth="1"/>
-    <col min="2" max="7" width="11.140625" style="5" bestFit="1" customWidth="1"/>
-    <col min="8" max="10" width="11.140625" style="5" customWidth="1"/>
-    <col min="11" max="13" width="11.140625" style="5" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="12.140625" style="5" bestFit="1" customWidth="1"/>
-    <col min="15" max="16384" width="10.85546875" style="5"/>
+    <col min="1" max="1" width="43.5" style="5" bestFit="1" customWidth="1"/>
+    <col min="2" max="7" width="11.1640625" style="5" bestFit="1" customWidth="1"/>
+    <col min="8" max="10" width="11.1640625" style="5" customWidth="1"/>
+    <col min="11" max="13" width="11.1640625" style="5" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="12.1640625" style="5" bestFit="1" customWidth="1"/>
+    <col min="15" max="16384" width="10.83203125" style="5"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16">
+    <row r="1" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A1" s="31" t="s">
         <v>33</v>
       </c>
@@ -6451,7 +6453,7 @@
         <v>447756</v>
       </c>
     </row>
-    <row r="3" spans="1:16">
+    <row r="3" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A3" s="1"/>
       <c r="B3" s="2" t="s">
         <v>8</v>
@@ -6493,7 +6495,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="4" spans="1:16">
+    <row r="4" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A4" s="49" t="s">
         <v>21</v>
       </c>
@@ -6536,7 +6538,7 @@
         <v>162308</v>
       </c>
     </row>
-    <row r="5" spans="1:16">
+    <row r="5" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A5" s="11" t="s">
         <v>22</v>
       </c>
@@ -6590,7 +6592,7 @@
       </c>
       <c r="N5" s="71"/>
     </row>
-    <row r="6" spans="1:16">
+    <row r="6" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A6" s="6" t="s">
         <v>23</v>
       </c>
@@ -6631,7 +6633,7 @@
       <c r="N6" s="70"/>
       <c r="P6" s="112"/>
     </row>
-    <row r="7" spans="1:16">
+    <row r="7" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A7" s="6"/>
       <c r="B7" s="8">
         <f>-'FY24'!M6+FY25_PB!B6</f>
@@ -6681,7 +6683,7 @@
       <c r="N7" s="70"/>
       <c r="P7" s="112"/>
     </row>
-    <row r="8" spans="1:16">
+    <row r="8" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A8" s="11" t="s">
         <v>34</v>
       </c>
@@ -6729,7 +6731,7 @@
         <v>417033.67</v>
       </c>
     </row>
-    <row r="9" spans="1:16">
+    <row r="9" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A9" s="6" t="s">
         <v>35</v>
       </c>
@@ -6786,61 +6788,61 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="10" spans="1:16">
+    <row r="10" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A10" s="11" t="s">
         <v>30</v>
       </c>
       <c r="B10" s="56">
-        <f>B6/B5</f>
+        <f t="shared" ref="B10:M10" si="3">B6/B5</f>
         <v>0.58202916698150886</v>
       </c>
       <c r="C10" s="56">
-        <f>C6/C5</f>
+        <f t="shared" si="3"/>
         <v>0.6108246353483896</v>
       </c>
       <c r="D10" s="56">
-        <f>D6/D5</f>
+        <f t="shared" si="3"/>
         <v>0.59620207882027942</v>
       </c>
       <c r="E10" s="56">
-        <f>E6/E5</f>
+        <f t="shared" si="3"/>
         <v>0.58126124956815017</v>
       </c>
       <c r="F10" s="56">
-        <f>F6/F5</f>
+        <f t="shared" si="3"/>
         <v>0.54607480690148735</v>
       </c>
       <c r="G10" s="56">
-        <f>G6/G5</f>
+        <f t="shared" si="3"/>
         <v>0.54905719576268575</v>
       </c>
       <c r="H10" s="56">
-        <f>H6/H5</f>
+        <f t="shared" si="3"/>
         <v>0.55287298253077721</v>
       </c>
       <c r="I10" s="56">
-        <f>I6/I5</f>
+        <f t="shared" si="3"/>
         <v>0.55645812724516164</v>
       </c>
       <c r="J10" s="56">
-        <f>J6/J5</f>
+        <f t="shared" si="3"/>
         <v>0.55944157278852191</v>
       </c>
       <c r="K10" s="56">
-        <f>K6/K5</f>
+        <f t="shared" si="3"/>
         <v>0.56070568561872913</v>
       </c>
       <c r="L10" s="56">
-        <f>L6/L5</f>
+        <f t="shared" si="3"/>
         <v>0.55933311914815498</v>
       </c>
       <c r="M10" s="56">
-        <f>M6/M5</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="N10" s="69"/>
     </row>
-    <row r="11" spans="1:16">
+    <row r="11" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A11" s="6" t="s">
         <v>36</v>
       </c>
@@ -6883,7 +6885,7 @@
         <v>9427</v>
       </c>
     </row>
-    <row r="12" spans="1:16">
+    <row r="12" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A12" s="23" t="s">
         <v>37</v>
       </c>
@@ -6923,7 +6925,7 @@
       <c r="M12" s="39"/>
       <c r="N12" s="76"/>
     </row>
-    <row r="13" spans="1:16">
+    <row r="13" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A13" s="27" t="s">
         <v>38</v>
       </c>
@@ -6936,11 +6938,11 @@
         <v>1408.7954333216744</v>
       </c>
       <c r="D13" s="28">
-        <f t="shared" ref="D13:L13" si="3">D9*D12</f>
+        <f t="shared" ref="D13:L13" si="4">D9*D12</f>
         <v>1355.9050555516667</v>
       </c>
       <c r="E13" s="28">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>1363.1583512846112</v>
       </c>
       <c r="F13" s="28">
@@ -6948,27 +6950,27 @@
         <v>1485.7849744679697</v>
       </c>
       <c r="G13" s="28">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>1401.6028003950544</v>
       </c>
       <c r="H13" s="28">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>1328.0801731351896</v>
       </c>
       <c r="I13" s="28">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>1525.8446513392421</v>
       </c>
       <c r="J13" s="28">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>613.63708460940711</v>
       </c>
       <c r="K13" s="28">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>1970.0560166357491</v>
       </c>
       <c r="L13" s="28">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>1248.2154383126876</v>
       </c>
       <c r="M13" s="28" t="e">
@@ -6980,7 +6982,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="15" spans="1:16">
+    <row r="15" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A15" s="52" t="s">
         <v>39</v>
       </c>
@@ -6989,15 +6991,15 @@
         <v>34034.009217746752</v>
       </c>
       <c r="C15" s="54">
-        <f t="shared" ref="C15:M15" si="4">C8-C13</f>
+        <f t="shared" ref="C15:M15" si="5">C8-C13</f>
         <v>38481.924566678324</v>
       </c>
       <c r="D15" s="54">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>37075.624944448333</v>
       </c>
       <c r="E15" s="54">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>37360.711648715391</v>
       </c>
       <c r="F15" s="54">
@@ -7005,35 +7007,35 @@
         <v>38599.515025532033</v>
       </c>
       <c r="G15" s="54">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>36908.747199604943</v>
       </c>
       <c r="H15" s="54">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>35393.689826864807</v>
       </c>
       <c r="I15" s="54">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>40715.855348660756</v>
       </c>
       <c r="J15" s="54">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>16403.862915390593</v>
       </c>
       <c r="K15" s="54">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>53247.17398336425</v>
       </c>
       <c r="L15" s="54">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>33764.304561687313</v>
       </c>
       <c r="M15" s="54" t="e">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="17" spans="1:20">
+    <row r="17" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A17" s="5" t="s">
         <v>40</v>
       </c>
@@ -7077,20 +7079,20 @@
       </c>
       <c r="M17" s="58"/>
     </row>
-    <row r="18" spans="1:20">
+    <row r="18" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A18" s="5" t="s">
         <v>41</v>
       </c>
       <c r="B18" s="55">
-        <f t="shared" ref="B18:M18" si="5">B8-B17</f>
+        <f t="shared" ref="B18:M18" si="6">B8-B17</f>
         <v>33190.53</v>
       </c>
       <c r="C18" s="55">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>37420.800000000003</v>
       </c>
       <c r="D18" s="55">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>36054.639999999999</v>
       </c>
       <c r="E18" s="55">
@@ -7098,7 +7100,7 @@
         <v>36326.240000000005</v>
       </c>
       <c r="F18" s="55">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>37603.370000000003</v>
       </c>
       <c r="G18" s="55">
@@ -7106,31 +7108,31 @@
         <v>35938.299999999996</v>
       </c>
       <c r="H18" s="55">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>34448.1</v>
       </c>
       <c r="I18" s="55">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>39626.259999999995</v>
       </c>
       <c r="J18" s="55">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>15962.02</v>
       </c>
       <c r="K18" s="55">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>51794.52</v>
       </c>
       <c r="L18" s="55">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>32840.870000000003</v>
       </c>
       <c r="M18" s="55">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:20">
+    <row r="19" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A19" s="5" t="s">
         <v>42</v>
       </c>
@@ -7139,15 +7141,15 @@
         <v>31843.359217746751</v>
       </c>
       <c r="C19" s="55">
-        <f t="shared" ref="C19:M19" si="6">C18-C13</f>
+        <f t="shared" ref="C19:M19" si="7">C18-C13</f>
         <v>36012.004566678326</v>
       </c>
       <c r="D19" s="55">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>34698.734944448333</v>
       </c>
       <c r="E19" s="55">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>34963.081648715393</v>
       </c>
       <c r="F19" s="55">
@@ -7155,7 +7157,7 @@
         <v>36117.585025532033</v>
       </c>
       <c r="G19" s="55">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>34536.69719960494</v>
       </c>
       <c r="H19" s="55">
@@ -7167,58 +7169,58 @@
         <v>38100.415348660754</v>
       </c>
       <c r="J19" s="55">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>15348.382915390594</v>
       </c>
       <c r="K19" s="55">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>49824.46398336425</v>
       </c>
       <c r="L19" s="55">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>31592.654561687315</v>
       </c>
       <c r="M19" s="55" t="e">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="20" spans="1:20">
+    <row r="20" spans="1:20" x14ac:dyDescent="0.2">
       <c r="G20" s="34"/>
       <c r="P20" s="58"/>
       <c r="R20" s="58"/>
       <c r="T20" s="55"/>
     </row>
-    <row r="21" spans="1:20">
+    <row r="21" spans="1:20" x14ac:dyDescent="0.2">
       <c r="C21" s="60"/>
       <c r="G21" s="38"/>
       <c r="I21" s="58"/>
       <c r="J21" s="58"/>
       <c r="K21" s="58"/>
     </row>
-    <row r="22" spans="1:20">
+    <row r="22" spans="1:20" x14ac:dyDescent="0.2">
       <c r="C22" s="60"/>
       <c r="I22" s="58"/>
       <c r="J22" s="58"/>
       <c r="K22" s="58"/>
     </row>
-    <row r="24" spans="1:20">
+    <row r="24" spans="1:20" x14ac:dyDescent="0.2">
       <c r="B24" s="112">
         <f>L6-B6</f>
         <v>71636</v>
       </c>
       <c r="J24" s="55"/>
     </row>
-    <row r="25" spans="1:20">
+    <row r="25" spans="1:20" x14ac:dyDescent="0.2">
       <c r="B25" s="5">
         <v>246796</v>
       </c>
       <c r="I25" s="136"/>
     </row>
-    <row r="26" spans="1:20">
+    <row r="26" spans="1:20" x14ac:dyDescent="0.2">
       <c r="L26" s="144"/>
     </row>
-    <row r="27" spans="1:20">
+    <row r="27" spans="1:20" x14ac:dyDescent="0.2">
       <c r="I27" s="137"/>
     </row>
   </sheetData>
@@ -7231,17 +7233,17 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FEA1CA45-4EA6-E543-B4CA-B49E1CEA765C}">
   <dimension ref="A1:T26"/>
-  <sheetFormatPr defaultColWidth="10.85546875" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="43.42578125" style="5" bestFit="1" customWidth="1"/>
-    <col min="2" max="7" width="11.140625" style="5" bestFit="1" customWidth="1"/>
-    <col min="8" max="10" width="11.140625" style="5" customWidth="1"/>
-    <col min="11" max="13" width="11.140625" style="5" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="12.140625" style="5" bestFit="1" customWidth="1"/>
-    <col min="15" max="16384" width="10.85546875" style="5"/>
+    <col min="1" max="1" width="43.5" style="5" bestFit="1" customWidth="1"/>
+    <col min="2" max="7" width="11.1640625" style="5" bestFit="1" customWidth="1"/>
+    <col min="8" max="10" width="11.1640625" style="5" customWidth="1"/>
+    <col min="11" max="13" width="11.1640625" style="5" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="12.1640625" style="5" bestFit="1" customWidth="1"/>
+    <col min="15" max="16384" width="10.83203125" style="5"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" ht="15.95" thickBot="1">
+    <row r="1" spans="1:16" ht="16" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A1" s="31" t="s">
         <v>33</v>
       </c>
@@ -7250,8 +7252,8 @@
         <v>447756</v>
       </c>
     </row>
-    <row r="2" spans="1:16" ht="15.95" thickBot="1"/>
-    <row r="3" spans="1:16" ht="15.95" thickBot="1">
+    <row r="2" spans="1:16" ht="16" thickBot="1" x14ac:dyDescent="0.25"/>
+    <row r="3" spans="1:16" ht="16" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>
       <c r="B3" s="2" t="s">
         <v>8</v>
@@ -7293,7 +7295,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="4" spans="1:16">
+    <row r="4" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A4" s="49" t="s">
         <v>21</v>
       </c>
@@ -7330,13 +7332,15 @@
       <c r="L4" s="42">
         <v>12064</v>
       </c>
-      <c r="M4" s="7"/>
+      <c r="M4" s="7">
+        <v>19158</v>
+      </c>
       <c r="N4" s="70">
         <f>SUM(B4:M4)</f>
-        <v>162308</v>
-      </c>
-    </row>
-    <row r="5" spans="1:16">
+        <v>181466</v>
+      </c>
+    </row>
+    <row r="5" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A5" s="11" t="s">
         <v>22</v>
       </c>
@@ -7386,11 +7390,11 @@
       </c>
       <c r="M5" s="13">
         <f t="shared" si="0"/>
-        <v>610064</v>
+        <v>629222</v>
       </c>
       <c r="N5" s="71"/>
     </row>
-    <row r="6" spans="1:16">
+    <row r="6" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A6" s="6" t="s">
         <v>23</v>
       </c>
@@ -7427,11 +7431,13 @@
       <c r="L6" s="9">
         <v>341229</v>
       </c>
-      <c r="M6" s="8"/>
+      <c r="M6" s="8">
+        <v>349395</v>
+      </c>
       <c r="N6" s="70"/>
       <c r="P6" s="112"/>
     </row>
-    <row r="7" spans="1:16">
+    <row r="7" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A7" s="11" t="s">
         <v>34</v>
       </c>
@@ -7473,13 +7479,15 @@
         <f>1231.23+33781.29</f>
         <v>35012.520000000004</v>
       </c>
-      <c r="M7" s="15"/>
+      <c r="M7" s="152">
+        <v>45550.48</v>
+      </c>
       <c r="N7" s="72">
         <f>SUM(B7:M7)</f>
-        <v>417033.67</v>
-      </c>
-    </row>
-    <row r="8" spans="1:16">
+        <v>462584.14999999997</v>
+      </c>
+    </row>
+    <row r="8" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A8" s="6" t="s">
         <v>35</v>
       </c>
@@ -7527,70 +7535,70 @@
         <f t="shared" si="1"/>
         <v>0.10260710549220613</v>
       </c>
-      <c r="M8" s="18" t="e">
+      <c r="M8" s="18">
         <f>M7/M6</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="N8" s="73" t="e">
+        <v>0.13036958170551954</v>
+      </c>
+      <c r="N8" s="73">
         <f>N7/M6</f>
-        <v>#DIV/0!</v>
-      </c>
-    </row>
-    <row r="9" spans="1:16">
+        <v>1.3239575552025644</v>
+      </c>
+    </row>
+    <row r="9" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A9" s="11" t="s">
         <v>30</v>
       </c>
       <c r="B9" s="56">
-        <f>B6/B5</f>
+        <f t="shared" ref="B9:M9" si="2">B6/B5</f>
         <v>0.58202916698150886</v>
       </c>
       <c r="C9" s="56">
-        <f>C6/C5</f>
+        <f t="shared" si="2"/>
         <v>0.6108246353483896</v>
       </c>
       <c r="D9" s="56">
-        <f>D6/D5</f>
+        <f t="shared" si="2"/>
         <v>0.59620207882027942</v>
       </c>
       <c r="E9" s="56">
-        <f>E6/E5</f>
+        <f t="shared" si="2"/>
         <v>0.58126124956815017</v>
       </c>
       <c r="F9" s="56">
-        <f>F6/F5</f>
+        <f t="shared" si="2"/>
         <v>0.54607480690148735</v>
       </c>
       <c r="G9" s="56">
-        <f>G6/G5</f>
+        <f t="shared" si="2"/>
         <v>0.54905719576268575</v>
       </c>
       <c r="H9" s="56">
-        <f>H6/H5</f>
+        <f t="shared" si="2"/>
         <v>0.55287298253077721</v>
       </c>
       <c r="I9" s="56">
-        <f>I6/I5</f>
+        <f t="shared" si="2"/>
         <v>0.55645812724516164</v>
       </c>
       <c r="J9" s="56">
-        <f>J6/J5</f>
+        <f t="shared" si="2"/>
         <v>0.55944157278852191</v>
       </c>
       <c r="K9" s="56">
-        <f>K6/K5</f>
+        <f t="shared" si="2"/>
         <v>0.56070568561872913</v>
       </c>
       <c r="L9" s="56">
-        <f>L6/L5</f>
+        <f t="shared" si="2"/>
         <v>0.55933311914815498</v>
       </c>
       <c r="M9" s="56">
-        <f>M6/M5</f>
-        <v>0</v>
+        <f t="shared" si="2"/>
+        <v>0.55528096601835286</v>
       </c>
       <c r="N9" s="69"/>
     </row>
-    <row r="10" spans="1:16">
+    <row r="10" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A10" s="6" t="s">
         <v>36</v>
       </c>
@@ -7627,13 +7635,15 @@
       <c r="L10" s="57">
         <v>1014</v>
       </c>
-      <c r="M10" s="57"/>
+      <c r="M10" s="57">
+        <v>921</v>
+      </c>
       <c r="N10" s="75">
         <f>SUM(B10:M10)</f>
-        <v>9427</v>
-      </c>
-    </row>
-    <row r="11" spans="1:16" ht="15.95" thickBot="1">
+        <v>10348</v>
+      </c>
+    </row>
+    <row r="11" spans="1:16" ht="16" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A11" s="23" t="s">
         <v>37</v>
       </c>
@@ -7670,10 +7680,12 @@
       <c r="L11" s="39">
         <v>12165</v>
       </c>
-      <c r="M11" s="39"/>
+      <c r="M11" s="39">
+        <v>12459</v>
+      </c>
       <c r="N11" s="76"/>
     </row>
-    <row r="12" spans="1:16" ht="17.100000000000001" thickTop="1" thickBot="1">
+    <row r="12" spans="1:16" ht="17" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A12" s="27" t="s">
         <v>38</v>
       </c>
@@ -7686,11 +7698,11 @@
         <v>1408.7954333216744</v>
       </c>
       <c r="D12" s="28">
-        <f t="shared" ref="D12:L12" si="2">D8*D11</f>
+        <f t="shared" ref="D12:L12" si="3">D8*D11</f>
         <v>1355.9050555516667</v>
       </c>
       <c r="E12" s="28">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>1363.1583512846112</v>
       </c>
       <c r="F12" s="28">
@@ -7698,39 +7710,39 @@
         <v>1485.7849744679697</v>
       </c>
       <c r="G12" s="28">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>1401.6028003950544</v>
       </c>
       <c r="H12" s="28">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>1328.0801731351896</v>
       </c>
       <c r="I12" s="28">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>1525.8446513392421</v>
       </c>
       <c r="J12" s="28">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>613.63708460940711</v>
       </c>
       <c r="K12" s="28">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>1970.0560166357491</v>
       </c>
       <c r="L12" s="28">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>1248.2154383126876</v>
       </c>
-      <c r="M12" s="28" t="e">
+      <c r="M12" s="28">
         <f>M8*M11</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="N12" s="77" t="e">
+        <v>1624.2746184690679</v>
+      </c>
+      <c r="N12" s="77">
         <f>SUM(B12:M12)</f>
-        <v>#DIV/0!</v>
-      </c>
-    </row>
-    <row r="14" spans="1:16">
+        <v>16672.525379775569</v>
+      </c>
+    </row>
+    <row r="14" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A14" s="52" t="s">
         <v>39</v>
       </c>
@@ -7739,15 +7751,15 @@
         <v>34034.009217746752</v>
       </c>
       <c r="C14" s="54">
-        <f t="shared" ref="C14:M14" si="3">C7-C12</f>
+        <f t="shared" ref="C14:M14" si="4">C7-C12</f>
         <v>38481.924566678324</v>
       </c>
       <c r="D14" s="54">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>37075.624944448333</v>
       </c>
       <c r="E14" s="54">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>37360.711648715391</v>
       </c>
       <c r="F14" s="54">
@@ -7755,35 +7767,35 @@
         <v>38599.515025532033</v>
       </c>
       <c r="G14" s="54">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>36908.747199604943</v>
       </c>
       <c r="H14" s="54">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>35393.689826864807</v>
       </c>
       <c r="I14" s="54">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>40715.855348660756</v>
       </c>
       <c r="J14" s="54">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>16403.862915390593</v>
       </c>
       <c r="K14" s="54">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>53247.17398336425</v>
       </c>
       <c r="L14" s="54">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>33764.304561687313</v>
       </c>
-      <c r="M14" s="54" t="e">
-        <f t="shared" si="3"/>
-        <v>#DIV/0!</v>
-      </c>
-    </row>
-    <row r="16" spans="1:16">
+      <c r="M14" s="54">
+        <f t="shared" si="4"/>
+        <v>43926.205381530934</v>
+      </c>
+    </row>
+    <row r="16" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A16" s="5" t="s">
         <v>40</v>
       </c>
@@ -7827,20 +7839,20 @@
       </c>
       <c r="M16" s="58"/>
     </row>
-    <row r="17" spans="1:20">
+    <row r="17" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A17" s="5" t="s">
         <v>41</v>
       </c>
       <c r="B17" s="55">
-        <f t="shared" ref="B17:M17" si="4">B7-B16</f>
+        <f t="shared" ref="B17:M17" si="5">B7-B16</f>
         <v>33190.53</v>
       </c>
       <c r="C17" s="55">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>37420.800000000003</v>
       </c>
       <c r="D17" s="55">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>36054.639999999999</v>
       </c>
       <c r="E17" s="55">
@@ -7848,7 +7860,7 @@
         <v>36326.240000000005</v>
       </c>
       <c r="F17" s="55">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>37603.370000000003</v>
       </c>
       <c r="G17" s="55">
@@ -7856,31 +7868,31 @@
         <v>35938.299999999996</v>
       </c>
       <c r="H17" s="55">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>34448.1</v>
       </c>
       <c r="I17" s="55">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>39626.259999999995</v>
       </c>
       <c r="J17" s="55">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>15962.02</v>
       </c>
       <c r="K17" s="55">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>51794.52</v>
       </c>
       <c r="L17" s="55">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>32840.870000000003</v>
       </c>
       <c r="M17" s="55">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="18" spans="1:20">
+        <f t="shared" si="5"/>
+        <v>45550.48</v>
+      </c>
+    </row>
+    <row r="18" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A18" s="5" t="s">
         <v>42</v>
       </c>
@@ -7889,15 +7901,15 @@
         <v>31843.359217746751</v>
       </c>
       <c r="C18" s="55">
-        <f t="shared" ref="C18:M18" si="5">C17-C12</f>
+        <f t="shared" ref="C18:M18" si="6">C17-C12</f>
         <v>36012.004566678326</v>
       </c>
       <c r="D18" s="55">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>34698.734944448333</v>
       </c>
       <c r="E18" s="55">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>34963.081648715393</v>
       </c>
       <c r="F18" s="55">
@@ -7905,7 +7917,7 @@
         <v>36117.585025532033</v>
       </c>
       <c r="G18" s="55">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>34536.69719960494</v>
       </c>
       <c r="H18" s="55">
@@ -7917,51 +7929,51 @@
         <v>38100.415348660754</v>
       </c>
       <c r="J18" s="55">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>15348.382915390594</v>
       </c>
       <c r="K18" s="55">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>49824.46398336425</v>
       </c>
       <c r="L18" s="55">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>31592.654561687315</v>
       </c>
-      <c r="M18" s="55" t="e">
-        <f t="shared" si="5"/>
-        <v>#DIV/0!</v>
-      </c>
-    </row>
-    <row r="19" spans="1:20">
+      <c r="M18" s="55">
+        <f t="shared" si="6"/>
+        <v>43926.205381530934</v>
+      </c>
+    </row>
+    <row r="19" spans="1:20" x14ac:dyDescent="0.2">
       <c r="G19" s="34"/>
       <c r="P19" s="58"/>
       <c r="R19" s="58"/>
       <c r="T19" s="55"/>
     </row>
-    <row r="20" spans="1:20">
+    <row r="20" spans="1:20" x14ac:dyDescent="0.2">
       <c r="C20" s="60"/>
       <c r="G20" s="38"/>
       <c r="I20" s="58"/>
       <c r="J20" s="58"/>
       <c r="K20" s="58"/>
     </row>
-    <row r="21" spans="1:20">
+    <row r="21" spans="1:20" x14ac:dyDescent="0.2">
       <c r="C21" s="60"/>
       <c r="I21" s="58"/>
       <c r="J21" s="58"/>
       <c r="K21" s="58"/>
     </row>
-    <row r="23" spans="1:20">
+    <row r="23" spans="1:20" x14ac:dyDescent="0.2">
       <c r="J23" s="55"/>
     </row>
-    <row r="24" spans="1:20">
+    <row r="24" spans="1:20" x14ac:dyDescent="0.2">
       <c r="I24" s="136"/>
     </row>
-    <row r="25" spans="1:20">
+    <row r="25" spans="1:20" x14ac:dyDescent="0.2">
       <c r="L25" s="144"/>
     </row>
-    <row r="26" spans="1:20">
+    <row r="26" spans="1:20" x14ac:dyDescent="0.2">
       <c r="I26" s="137"/>
     </row>
   </sheetData>
@@ -7974,19 +7986,19 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EEF543C9-DA1C-7340-BBE5-B6E66BB1F9AE}">
   <dimension ref="A1:T21"/>
-  <sheetFormatPr defaultColWidth="10.85546875" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="56.42578125" style="5" customWidth="1"/>
-    <col min="2" max="7" width="11.140625" style="5" bestFit="1" customWidth="1"/>
-    <col min="8" max="10" width="11.140625" style="5" customWidth="1"/>
-    <col min="11" max="13" width="11.140625" style="5" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="12.140625" style="5" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="10.85546875" style="5"/>
-    <col min="16" max="16" width="11.140625" style="5" bestFit="1" customWidth="1"/>
-    <col min="17" max="16384" width="10.85546875" style="5"/>
+    <col min="1" max="1" width="56.5" style="5" customWidth="1"/>
+    <col min="2" max="7" width="11.1640625" style="5" bestFit="1" customWidth="1"/>
+    <col min="8" max="10" width="11.1640625" style="5" customWidth="1"/>
+    <col min="11" max="13" width="11.1640625" style="5" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="12.1640625" style="5" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="10.83203125" style="5"/>
+    <col min="16" max="16" width="11.1640625" style="5" bestFit="1" customWidth="1"/>
+    <col min="17" max="16384" width="10.83203125" style="5"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" ht="15.95" thickBot="1">
+    <row r="1" spans="1:16" ht="16" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A1" s="31" t="s">
         <v>33</v>
       </c>
@@ -7995,8 +8007,8 @@
         <v>288980</v>
       </c>
     </row>
-    <row r="2" spans="1:16" ht="15.95" thickBot="1"/>
-    <row r="3" spans="1:16" ht="15.95" thickBot="1">
+    <row r="2" spans="1:16" ht="16" thickBot="1" x14ac:dyDescent="0.25"/>
+    <row r="3" spans="1:16" ht="16" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>
       <c r="B3" s="2" t="s">
         <v>8</v>
@@ -8039,7 +8051,7 @@
       </c>
       <c r="P3" s="35"/>
     </row>
-    <row r="4" spans="1:16">
+    <row r="4" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A4" s="49" t="s">
         <v>21</v>
       </c>
@@ -8085,7 +8097,7 @@
       </c>
       <c r="P4" s="35"/>
     </row>
-    <row r="5" spans="1:16">
+    <row r="5" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A5" s="11" t="s">
         <v>22</v>
       </c>
@@ -8139,7 +8151,7 @@
       </c>
       <c r="N5" s="71"/>
     </row>
-    <row r="6" spans="1:16">
+    <row r="6" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A6" s="6" t="s">
         <v>23</v>
       </c>
@@ -8182,7 +8194,7 @@
       <c r="N6" s="70"/>
       <c r="P6" s="112"/>
     </row>
-    <row r="7" spans="1:16">
+    <row r="7" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A7" s="11" t="s">
         <v>34</v>
       </c>
@@ -8227,7 +8239,7 @@
         <v>499270.30000000005</v>
       </c>
     </row>
-    <row r="8" spans="1:16">
+    <row r="8" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A8" s="6" t="s">
         <v>35</v>
       </c>
@@ -8284,7 +8296,7 @@
         <v>2.0230080714436216</v>
       </c>
     </row>
-    <row r="9" spans="1:16">
+    <row r="9" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A9" s="11" t="s">
         <v>30</v>
       </c>
@@ -8338,7 +8350,7 @@
       </c>
       <c r="N9" s="69"/>
     </row>
-    <row r="10" spans="1:16">
+    <row r="10" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A10" s="6" t="s">
         <v>36</v>
       </c>
@@ -8383,7 +8395,7 @@
         <v>7851</v>
       </c>
     </row>
-    <row r="11" spans="1:16" ht="15.95" thickBot="1">
+    <row r="11" spans="1:16" ht="16" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A11" s="23" t="s">
         <v>37</v>
       </c>
@@ -8427,7 +8439,7 @@
       </c>
       <c r="N11" s="76"/>
     </row>
-    <row r="12" spans="1:16" ht="17.100000000000001" thickTop="1" thickBot="1">
+    <row r="12" spans="1:16" ht="17" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A12" s="27" t="s">
         <v>38</v>
       </c>
@@ -8484,7 +8496,7 @@
         <v>24236.725104646648</v>
       </c>
     </row>
-    <row r="14" spans="1:16">
+    <row r="14" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A14" s="52" t="s">
         <v>39</v>
       </c>
@@ -8537,7 +8549,7 @@
         <v>32256.633393977212</v>
       </c>
     </row>
-    <row r="16" spans="1:16">
+    <row r="16" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A16" s="5" t="s">
         <v>40</v>
       </c>
@@ -8578,7 +8590,7 @@
         <v>2082.16</v>
       </c>
     </row>
-    <row r="17" spans="1:20">
+    <row r="17" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A17" s="5" t="s">
         <v>41</v>
       </c>
@@ -8631,7 +8643,7 @@
         <v>31545.49</v>
       </c>
     </row>
-    <row r="18" spans="1:20">
+    <row r="18" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A18" s="5" t="s">
         <v>42</v>
       </c>
@@ -8684,13 +8696,13 @@
         <v>30174.473393977212</v>
       </c>
     </row>
-    <row r="19" spans="1:20">
+    <row r="19" spans="1:20" x14ac:dyDescent="0.2">
       <c r="G19" s="34"/>
       <c r="P19" s="58"/>
       <c r="R19" s="58"/>
       <c r="T19" s="55"/>
     </row>
-    <row r="20" spans="1:20">
+    <row r="20" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A20" s="5" t="s">
         <v>44</v>
       </c>
@@ -8703,7 +8715,7 @@
       <c r="J20" s="58"/>
       <c r="K20" s="58"/>
     </row>
-    <row r="21" spans="1:20">
+    <row r="21" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A21" s="5" t="s">
         <v>45</v>
       </c>
@@ -8725,16 +8737,16 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{380343CA-8DB1-784E-A735-7745B871B90B}">
   <dimension ref="A1:M23"/>
-  <sheetFormatPr defaultColWidth="10.85546875" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="47.28515625" style="5" bestFit="1" customWidth="1"/>
-    <col min="2" max="7" width="11.140625" style="5" bestFit="1" customWidth="1"/>
-    <col min="8" max="10" width="11.140625" style="5" customWidth="1"/>
-    <col min="11" max="13" width="11.140625" style="5" bestFit="1" customWidth="1"/>
-    <col min="14" max="16384" width="10.85546875" style="5"/>
+    <col min="1" max="1" width="47.33203125" style="5" bestFit="1" customWidth="1"/>
+    <col min="2" max="7" width="11.1640625" style="5" bestFit="1" customWidth="1"/>
+    <col min="8" max="10" width="11.1640625" style="5" customWidth="1"/>
+    <col min="11" max="13" width="11.1640625" style="5" bestFit="1" customWidth="1"/>
+    <col min="14" max="16384" width="10.83203125" style="5"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" ht="15.95" thickBot="1">
+    <row r="1" spans="1:13" ht="16" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A1" s="31" t="s">
         <v>33</v>
       </c>
@@ -8743,7 +8755,7 @@
         <v>182477</v>
       </c>
     </row>
-    <row r="2" spans="1:13" ht="15.95" thickBot="1">
+    <row r="2" spans="1:13" ht="16" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A2" s="31" t="s">
         <v>46</v>
       </c>
@@ -8752,8 +8764,8 @@
         <v>1941</v>
       </c>
     </row>
-    <row r="3" spans="1:13" ht="15.95" thickBot="1"/>
-    <row r="4" spans="1:13" ht="15.95" thickBot="1">
+    <row r="3" spans="1:13" ht="16" thickBot="1" x14ac:dyDescent="0.25"/>
+    <row r="4" spans="1:13" ht="16" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A4" s="1"/>
       <c r="B4" s="2" t="s">
         <v>8</v>
@@ -8792,7 +8804,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="5" spans="1:13">
+    <row r="5" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A5" s="49" t="s">
         <v>47</v>
       </c>
@@ -8833,7 +8845,7 @@
         <v>11223</v>
       </c>
     </row>
-    <row r="6" spans="1:13">
+    <row r="6" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A6" s="11" t="s">
         <v>22</v>
       </c>
@@ -8886,7 +8898,7 @@
         <v>288980</v>
       </c>
     </row>
-    <row r="7" spans="1:13">
+    <row r="7" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A7" s="6" t="s">
         <v>23</v>
       </c>
@@ -8927,7 +8939,7 @@
         <v>149689</v>
       </c>
     </row>
-    <row r="8" spans="1:13">
+    <row r="8" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A8" s="11" t="s">
         <v>34</v>
       </c>
@@ -8968,7 +8980,7 @@
         <v>35050.03</v>
       </c>
     </row>
-    <row r="9" spans="1:13">
+    <row r="9" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A9" s="6" t="s">
         <v>48</v>
       </c>
@@ -9009,7 +9021,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:13">
+    <row r="10" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A10" s="11" t="s">
         <v>35</v>
       </c>
@@ -9062,7 +9074,7 @@
         <v>0.2341523425234987</v>
       </c>
     </row>
-    <row r="11" spans="1:13">
+    <row r="11" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A11" s="6" t="s">
         <v>30</v>
       </c>
@@ -9115,7 +9127,7 @@
         <v>0.51799086441968301</v>
       </c>
     </row>
-    <row r="12" spans="1:13">
+    <row r="12" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A12" s="11" t="s">
         <v>36</v>
       </c>
@@ -9156,7 +9168,7 @@
         <v>439</v>
       </c>
     </row>
-    <row r="13" spans="1:13" ht="15.95" thickBot="1">
+    <row r="13" spans="1:13" ht="16" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A13" s="45" t="s">
         <v>37</v>
       </c>
@@ -9206,7 +9218,7 @@
         <v>9133</v>
       </c>
     </row>
-    <row r="14" spans="1:13" ht="17.100000000000001" thickTop="1" thickBot="1">
+    <row r="14" spans="1:13" ht="17" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A14" s="27" t="s">
         <v>38</v>
       </c>
@@ -9259,7 +9271,7 @@
         <v>2138.5133442671136</v>
       </c>
     </row>
-    <row r="16" spans="1:13">
+    <row r="16" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A16" s="52" t="s">
         <v>39</v>
       </c>
@@ -9291,17 +9303,17 @@
         <v>32911.516655732885</v>
       </c>
     </row>
-    <row r="17" spans="1:13">
+    <row r="17" spans="1:13" x14ac:dyDescent="0.2">
       <c r="B17" s="59"/>
     </row>
-    <row r="18" spans="1:13">
+    <row r="18" spans="1:13" x14ac:dyDescent="0.2">
       <c r="L18" s="55">
         <f>L16-1958.75</f>
         <v>27804.833491433033</v>
       </c>
       <c r="M18" s="55"/>
     </row>
-    <row r="21" spans="1:13">
+    <row r="21" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A21" s="5" t="s">
         <v>49</v>
       </c>
@@ -9354,10 +9366,10 @@
         <v>35050.03</v>
       </c>
     </row>
-    <row r="22" spans="1:13">
+    <row r="22" spans="1:13" x14ac:dyDescent="0.2">
       <c r="G22" s="38"/>
     </row>
-    <row r="23" spans="1:13">
+    <row r="23" spans="1:13" x14ac:dyDescent="0.2">
       <c r="K23" s="5" t="s">
         <v>50</v>
       </c>
@@ -9371,18 +9383,18 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2A882FF9-E67B-BD4A-BCB1-2A8FD335EAF2}">
   <dimension ref="A1:N21"/>
-  <sheetFormatPr defaultColWidth="10.85546875" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="41.28515625" style="5" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="9.85546875" style="5" customWidth="1"/>
-    <col min="3" max="6" width="10.140625" style="5" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="11.140625" style="5" bestFit="1" customWidth="1"/>
-    <col min="8" max="10" width="11.140625" style="5" customWidth="1"/>
-    <col min="11" max="13" width="11.140625" style="5" bestFit="1" customWidth="1"/>
-    <col min="14" max="16384" width="10.85546875" style="5"/>
+    <col min="1" max="1" width="41.33203125" style="5" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.83203125" style="5" customWidth="1"/>
+    <col min="3" max="6" width="10.1640625" style="5" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="11.1640625" style="5" bestFit="1" customWidth="1"/>
+    <col min="8" max="10" width="11.1640625" style="5" customWidth="1"/>
+    <col min="11" max="13" width="11.1640625" style="5" bestFit="1" customWidth="1"/>
+    <col min="14" max="16384" width="10.83203125" style="5"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" ht="15.95" thickBot="1">
+    <row r="1" spans="1:14" ht="16" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A1" s="31" t="s">
         <v>51</v>
       </c>
@@ -9390,8 +9402,8 @@
         <v>104017</v>
       </c>
     </row>
-    <row r="2" spans="1:14" ht="15.95" thickBot="1"/>
-    <row r="3" spans="1:14" ht="15.95" thickBot="1">
+    <row r="2" spans="1:14" ht="16" thickBot="1" x14ac:dyDescent="0.25"/>
+    <row r="3" spans="1:14" ht="16" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>
       <c r="B3" s="2" t="s">
         <v>8</v>
@@ -9430,7 +9442,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="4" spans="1:14" ht="15.95" thickBot="1">
+    <row r="4" spans="1:14" ht="16" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A4" s="6" t="s">
         <v>52</v>
       </c>
@@ -9471,7 +9483,7 @@
         <v>13537</v>
       </c>
     </row>
-    <row r="5" spans="1:14" ht="15.95" thickTop="1">
+    <row r="5" spans="1:14" ht="16" thickTop="1" x14ac:dyDescent="0.2">
       <c r="A5" s="11" t="s">
         <v>22</v>
       </c>
@@ -9524,7 +9536,7 @@
         <v>182477</v>
       </c>
     </row>
-    <row r="6" spans="1:14">
+    <row r="6" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A6" s="6" t="s">
         <v>53</v>
       </c>
@@ -9566,7 +9578,7 @@
       </c>
       <c r="N6" s="112"/>
     </row>
-    <row r="7" spans="1:14">
+    <row r="7" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A7" s="11" t="s">
         <v>34</v>
       </c>
@@ -9607,7 +9619,7 @@
         <v>15671.14</v>
       </c>
     </row>
-    <row r="8" spans="1:14">
+    <row r="8" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A8" s="6" t="s">
         <v>48</v>
       </c>
@@ -9648,7 +9660,7 @@
         <v>633.86</v>
       </c>
     </row>
-    <row r="9" spans="1:14">
+    <row r="9" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A9" s="11" t="s">
         <v>54</v>
       </c>
@@ -9701,7 +9713,7 @@
         <v>0.17179795170059425</v>
       </c>
     </row>
-    <row r="10" spans="1:14">
+    <row r="10" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A10" s="6" t="s">
         <v>30</v>
       </c>
@@ -9754,7 +9766,7 @@
         <v>0.52010938364835024</v>
       </c>
     </row>
-    <row r="11" spans="1:14" ht="15.95" thickBot="1">
+    <row r="11" spans="1:14" ht="16" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A11" s="23" t="s">
         <v>37</v>
       </c>
@@ -9806,7 +9818,7 @@
         <v>1941</v>
       </c>
     </row>
-    <row r="12" spans="1:14" ht="17.100000000000001" thickTop="1" thickBot="1">
+    <row r="12" spans="1:14" ht="17" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A12" s="27" t="s">
         <v>38</v>
       </c>
@@ -9859,7 +9871,7 @@
         <v>333.45982425085344</v>
       </c>
     </row>
-    <row r="14" spans="1:14">
+    <row r="14" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A14" s="5" t="s">
         <v>55</v>
       </c>
@@ -9873,7 +9885,7 @@
         <v>5105</v>
       </c>
     </row>
-    <row r="15" spans="1:14" ht="15.95">
+    <row r="15" spans="1:14" ht="16" x14ac:dyDescent="0.2">
       <c r="A15" s="36" t="s">
         <v>56</v>
       </c>
@@ -9891,7 +9903,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="17" spans="1:13">
+    <row r="17" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A17" s="5" t="s">
         <v>57</v>
       </c>
@@ -9944,13 +9956,13 @@
         <v>16305</v>
       </c>
     </row>
-    <row r="19" spans="1:13">
+    <row r="19" spans="1:13" x14ac:dyDescent="0.2">
       <c r="G19" s="34"/>
     </row>
-    <row r="20" spans="1:13">
+    <row r="20" spans="1:13" x14ac:dyDescent="0.2">
       <c r="G20" s="38"/>
     </row>
-    <row r="21" spans="1:13">
+    <row r="21" spans="1:13" x14ac:dyDescent="0.2">
       <c r="K21" s="5" t="s">
         <v>50</v>
       </c>
@@ -9964,13 +9976,13 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{64686866-CD2C-4344-B0B0-3972EF100116}">
   <dimension ref="B1:W7"/>
-  <sheetFormatPr defaultColWidth="10.85546875" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="2" max="2" width="38.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="38.83203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:23" ht="15.95" thickBot="1"/>
-    <row r="2" spans="2:23" ht="18.95">
+    <row r="1" spans="2:23" ht="16" thickBot="1" x14ac:dyDescent="0.25"/>
+    <row r="2" spans="2:23" ht="19" x14ac:dyDescent="0.25">
       <c r="B2" s="88"/>
       <c r="C2" s="145" t="s">
         <v>58</v>
@@ -9998,7 +10010,7 @@
       <c r="V2" s="146"/>
       <c r="W2" s="147"/>
     </row>
-    <row r="3" spans="2:23">
+    <row r="3" spans="2:23" x14ac:dyDescent="0.2">
       <c r="B3" s="89"/>
       <c r="C3" s="97" t="s">
         <v>60</v>
@@ -10064,7 +10076,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="4" spans="2:23">
+    <row r="4" spans="2:23" x14ac:dyDescent="0.2">
       <c r="B4" s="90" t="s">
         <v>36</v>
       </c>
@@ -10141,10 +10153,10 @@
       </c>
       <c r="W4" s="83">
         <f>'FY25'!M10</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5" spans="2:23">
+        <v>921</v>
+      </c>
+    </row>
+    <row r="5" spans="2:23" x14ac:dyDescent="0.2">
       <c r="B5" s="91" t="s">
         <v>37</v>
       </c>
@@ -10221,10 +10233,10 @@
       </c>
       <c r="W5" s="84">
         <f>'FY25'!M11</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6" spans="2:23">
+        <v>12459</v>
+      </c>
+    </row>
+    <row r="6" spans="2:23" x14ac:dyDescent="0.2">
       <c r="B6" s="90" t="s">
         <v>71</v>
       </c>
@@ -10307,10 +10319,10 @@
       </c>
       <c r="W6" s="101">
         <f t="shared" si="9"/>
-        <v>-12165</v>
-      </c>
-    </row>
-    <row r="7" spans="2:23" ht="15.95" thickBot="1">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="7" spans="2:23" ht="16" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B7" s="92" t="s">
         <v>72</v>
       </c>
@@ -10393,7 +10405,7 @@
       </c>
       <c r="W7" s="87">
         <f t="shared" ref="W7" si="20">W4-W6</f>
-        <v>12165</v>
+        <v>627</v>
       </c>
     </row>
   </sheetData>
@@ -10410,14 +10422,14 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{735F8B00-DF6F-E740-A737-9B65F0C9471C}">
   <dimension ref="A1:AW4"/>
-  <sheetFormatPr defaultColWidth="10.85546875" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="15.28515625" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="11.140625" bestFit="1" customWidth="1"/>
-    <col min="38" max="38" width="11.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="15.33203125" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="11.1640625" bestFit="1" customWidth="1"/>
+    <col min="38" max="38" width="11.1640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:49" ht="15.95" thickBot="1">
+    <row r="1" spans="1:49" ht="16" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B1" s="149" t="s">
         <v>73</v>
       </c>
@@ -10475,7 +10487,7 @@
       <c r="AV1" s="150"/>
       <c r="AW1" s="151"/>
     </row>
-    <row r="2" spans="1:49">
+    <row r="2" spans="1:49" x14ac:dyDescent="0.2">
       <c r="B2" s="61" t="s">
         <v>75</v>
       </c>
@@ -10621,7 +10633,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="3" spans="1:49">
+    <row r="3" spans="1:49" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>87</v>
       </c>
@@ -10791,10 +10803,10 @@
       </c>
       <c r="AW3" s="63">
         <f>'FY25'!M6</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="4" spans="1:49">
+        <v>349395</v>
+      </c>
+    </row>
+    <row r="4" spans="1:49" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>34</v>
       </c>
@@ -10964,7 +10976,7 @@
       </c>
       <c r="AW4" s="122">
         <f>'FY25'!M7</f>
-        <v>0</v>
+        <v>45550.48</v>
       </c>
     </row>
   </sheetData>

</xml_diff>